<commit_message>
Fix: integre la vraie consommation et gere les donnees manquantes
</commit_message>
<xml_diff>
--- a/data/matieres.xlsx
+++ b/data/matieres.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\israc\OneDrive\Documents\pilotage-stock-production\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59990CEA-30F6-4207-8568-F0E5FF3EC44A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A092A6A-6E63-4630-BBD0-3BE63EC5E841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="204">
   <si>
     <t>code_matiere</t>
   </si>
@@ -1254,7 +1254,9 @@
       <c r="B7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
@@ -1280,7 +1282,9 @@
       <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D8" s="3">
         <v>4</v>
       </c>
@@ -1306,7 +1310,9 @@
       <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D9" s="3">
         <v>5</v>
       </c>
@@ -1332,7 +1338,9 @@
       <c r="B10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D10" s="3">
         <v>4</v>
       </c>
@@ -1358,7 +1366,9 @@
       <c r="B11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D11" s="3">
         <v>1</v>
       </c>
@@ -1474,7 +1484,9 @@
       <c r="B15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D15" s="3">
         <v>3</v>
       </c>
@@ -1500,7 +1512,9 @@
       <c r="B16" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D16" s="3">
         <v>1</v>
       </c>
@@ -1526,7 +1540,9 @@
       <c r="B17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D17" s="3">
         <v>1</v>
       </c>
@@ -1552,7 +1568,9 @@
       <c r="B18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D18" s="3">
         <v>3</v>
       </c>
@@ -1578,7 +1596,9 @@
       <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D19" s="3">
         <v>3</v>
       </c>
@@ -1604,7 +1624,9 @@
       <c r="B20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D20" s="3">
         <v>4</v>
       </c>
@@ -1630,7 +1652,9 @@
       <c r="B21" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D21" s="3">
         <v>3</v>
       </c>
@@ -1656,7 +1680,9 @@
       <c r="B22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D22" s="3">
         <v>3</v>
       </c>
@@ -1682,7 +1708,9 @@
       <c r="B23" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D23" s="3">
         <v>3</v>
       </c>
@@ -1708,7 +1736,9 @@
       <c r="B24" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D24" s="3">
         <v>3</v>
       </c>
@@ -1734,7 +1764,9 @@
       <c r="B25" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D25" s="3">
         <v>4</v>
       </c>
@@ -1850,7 +1882,9 @@
       <c r="B29" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D29" s="3">
         <v>208</v>
       </c>
@@ -1906,7 +1940,9 @@
       <c r="B31" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D31" s="3">
         <v>85</v>
       </c>
@@ -2050,7 +2086,9 @@
       <c r="B36" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D36" s="3">
         <v>0</v>
       </c>
@@ -3272,7 +3310,9 @@
       <c r="B77" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C77" s="2"/>
+      <c r="C77" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D77" s="3">
         <v>0</v>
       </c>

</xml_diff>